<commit_message>
Fix template crash: strip images/comments from AsBuiltSubmittalFormBlank.xlsx
exceljs's DrawingXform.parseOpen() does literal string matching against
the namespace-PREFIXED tag 'xdr:wsDr', but openpyxl writes drawing XML
using the unprefixed default-namespace convention (<wsDr xmlns=...>).
exceljs never recognizes the root tag, leaves model.drawings['drawing1']
undefined, and then crashes in reconcile() with 'Cannot read properties
of undefined (reading anchors)' when loading the template.

The 2 embedded images and 8 cell comments on the template are cosmetic
only (title-block instructions) and aren't needed for the auto-filled
data, so the fix strips them from the template via openpyxl instead of
trying to reconcile openpyxl/exceljs's differing XML conventions.

Verified: fillAsBuiltForm() + reload via a fresh ExcelJS.Workbook now
succeeds for 1-sheet, 3-sheet (pagination), and empty-rows cases.
</commit_message>
<xml_diff>
--- a/data/AsBuiltSubmittalFormBlank.xlsx
+++ b/data/AsBuiltSubmittalFormBlank.xlsx
@@ -599,147 +599,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>ell0zpi</author>
-  </authors>
-  <commentList>
-    <comment ref="B5" authorId="0" shapeId="0">
-      <text>
-        <t>Send the email to Project Control to create the As Built PCS #.
-If submitting only an Operating Diagram, send to Sam Fried.  
-(Cam Scanner App for iPhone or Android is recommended.
-iPhone Enhancement Settings: Auto Process=Magic Color, Image Size=Large, Image Quality=highest
-Android Settings/Scan Settings: Enhance Mode=Magic Color, Camera Settings=Highest Megapixel Available.)</t>
-      </text>
-    </comment>
-    <comment ref="B6" authorId="0" shapeId="0">
-      <text>
-        <t>Add Senders name (Construction Lead, Ops Lead or P&amp;C Engineer's name)</t>
-      </text>
-    </comment>
-    <comment ref="B7" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Enter the name of the P&amp;C or Substation project engineer who released the project.  This information can be found on the project release letter or in PUR.  Please communicate with the project engineer prior to making any as-built changes.  </t>
-      </text>
-    </comment>
-    <comment ref="G8" authorId="0" shapeId="0">
-      <text>
-        <t>Select Substation Area from Drop Down list.</t>
-      </text>
-    </comment>
-    <comment ref="G9" authorId="0" shapeId="0">
-      <text>
-        <t>Today's Date auto-populates.</t>
-      </text>
-    </comment>
-    <comment ref="E11" authorId="0" shapeId="0">
-      <text>
-        <t>Select As Built Cause from Drop Down list.</t>
-      </text>
-    </comment>
-    <comment ref="J11" authorId="0" shapeId="0">
-      <text>
-        <t>Select As Built Cause from Drop Down list.</t>
-      </text>
-    </comment>
-    <comment ref="B42" authorId="0" shapeId="0">
-      <text>
-        <t>Enter any comments or instructions you have about the project or as builts.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>152400</colOff>
-      <row>0</row>
-      <rowOff>47626</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>423429</colOff>
-      <row>3</row>
-      <rowOff>261572</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Picture 4"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="152400" y="47626"/>
-          <a:ext cx="904875" cy="692794"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>7</col>
-      <colOff>25976</colOff>
-      <row>0</row>
-      <rowOff>28576</rowOff>
-    </from>
-    <to>
-      <col>9</col>
-      <colOff>933449</colOff>
-      <row>3</row>
-      <rowOff>80020</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Picture 5"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="16200000">
-          <a:off x="5285764" y="-650553"/>
-          <a:ext cx="527694" cy="1885951"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -1924,8 +1783,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>